<commit_message>
chore: update roadmap, add Data Request, ignore Office lock files
- Refresh SkyportHome_Roadmap.xlsx with latest planning
- Add Data_Request-2.xlsx
- Ignore Excel/Word lock files (~$*) to keep them out of version control

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/SkyportHome_Roadmap.xlsx
+++ b/SkyportHome_Roadmap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vishwas/Documents/DevelopmentProjects/Skyport-Web/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71485852-8D22-0C4C-B322-C2ED43A701EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D50A3653-BC2C-7A4B-8712-803DD5059AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="49900" yWindow="1360" windowWidth="46280" windowHeight="25180" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16800" yWindow="500" windowWidth="30240" windowHeight="18880" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="2" r:id="rId1"/>

</xml_diff>